<commit_message>
sửa lại mail và thêm secure
</commit_message>
<xml_diff>
--- a/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
+++ b/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
@@ -8,29 +8,60 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\khanhmf\SURVEY\SURVEY\SURVEY\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C975574-4860-43C5-8E02-F9C1993D0AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A15EE23-E9C8-402F-8BFB-5DBCB6B165C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="評価シート" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+  <si>
+    <t>Kết quả khảo sát đánh giá 360 / 360度評価調査結果</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
   <si>
     <t>Tên nhân viên / 氏名</t>
   </si>
   <si>
+    <t>1. Hợp tác &amp; làm việc nhóm / チームワーク</t>
+  </si>
+  <si>
     <t>Nhóm / チーム</t>
   </si>
   <si>
+    <t>2. Giao tiếp &amp; chia sẻ thông tin / コミュニケーション</t>
+  </si>
+  <si>
     <t>Thời gian / 評価期間</t>
   </si>
   <si>
+    <t>3. Đào tạo &amp; hỗ trợ người khác / 指導・サポート</t>
+  </si>
+  <si>
+    <t>4. Trách nhiệm &amp; tự chủ / 責任感・主体性</t>
+  </si>
+  <si>
     <t>Nhóm / 評価項目</t>
   </si>
   <si>
@@ -49,25 +80,10 @@
     <t>Điểm cần cải thiện / 短所</t>
   </si>
   <si>
+    <t>5. Kỷ luật &amp; tuân thủ thời gian / 規律・時間遵守</t>
+  </si>
+  <si>
     <t>Nhận xét chung / 総合コメント</t>
-  </si>
-  <si>
-    <t>1. Hợp tác &amp; làm việc nhóm / チームワーク</t>
-  </si>
-  <si>
-    <t>2. Giao tiếp &amp; chia sẻ thông tin / コミュニケーション</t>
-  </si>
-  <si>
-    <t>3. Đào tạo &amp; hỗ trợ người khác / 指導・サポート</t>
-  </si>
-  <si>
-    <t>4. Trách nhiệm &amp; tự chủ / 責任感・主体性</t>
-  </si>
-  <si>
-    <t>5. Kỷ luật &amp; tuân thủ thời gian / 規律・時間遵守</t>
-  </si>
-  <si>
-    <t>Kết quả khảo sát đánh giá 360 / 360度評価調査結果</t>
   </si>
 </sst>
 </file>
@@ -139,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -150,12 +166,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -172,6 +193,493 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" b="1"/>
+              <a:t>Tổng hợp đánh </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="vi-VN" b="1"/>
+              <a:t>giá</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ja-JP" altLang="en-US" b="1"/>
+              <a:t>レビューの概要</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" b="1"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.9917592592592586E-2"/>
+          <c:y val="3.3629629629629627E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="1"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>評価シート!$N$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Điểm tốt / 長所</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="15875" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="38000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>評価シート!$M$2:$M$6</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1. Hợp tác &amp; làm việc nhóm / チームワーク</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2. Giao tiếp &amp; chia sẻ thông tin / コミュニケーション</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3. Đào tạo &amp; hỗ trợ người khác / 指導・サポート</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4. Trách nhiệm &amp; tự chủ / 責任感・主体性</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5. Kỷ luật &amp; tuân thủ thời gian / 規律・時間遵守</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>評価シート!$N$2:$N$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E379-4408-AE36-96FCAF2CD8BF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>評価シート!$O$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Điểm cần cải thiện / 短所</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="15875" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="38000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>評価シート!$M$2:$M$6</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1. Hợp tác &amp; làm việc nhóm / チームワーク</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2. Giao tiếp &amp; chia sẻ thông tin / コミュニケーション</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3. Đào tạo &amp; hỗ trợ người khác / 指導・サポート</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4. Trách nhiệm &amp; tự chủ / 責任感・主体性</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5. Kỷ luật &amp; tuân thủ thời gian / 規律・時間遵守</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>評価シート!$O$2:$O$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E379-4408-AE36-96FCAF2CD8BF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="10"/>
+        <c:axId val="100"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="10"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="100"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="10"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1985531</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>188286</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5400000" cy="3429000"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -459,92 +967,161 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="47.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" customWidth="1"/>
-    <col min="5" max="5" width="35.42578125" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" customWidth="1"/>
-    <col min="9" max="9" width="38.5703125" customWidth="1"/>
+    <col min="1" max="1" width="30" style="5" customWidth="1"/>
+    <col min="2" max="2" width="47.5703125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34.140625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="38.5703125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19" customWidth="1"/>
+    <col min="15" max="15" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:15" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="M1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2">
+        <f>$C7</f>
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <f>$G7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="M3" t="s">
+        <v>5</v>
+      </c>
+      <c r="N3" s="7">
+        <f t="shared" ref="N3:N6" si="0">$C8</f>
+        <v>0</v>
+      </c>
+      <c r="O3" s="7">
+        <f t="shared" ref="O3:O6" si="1">$G8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="M4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N4" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O4" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M5" t="s">
+        <v>8</v>
+      </c>
+      <c r="N5" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="N6" s="7">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="O6" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -555,9 +1132,9 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -568,9 +1145,9 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -581,9 +1158,9 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -594,9 +1171,9 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -607,51 +1184,51 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -663,5 +1240,6 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sua giao dien va file
</commit_message>
<xml_diff>
--- a/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
+++ b/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\khanhmf\SURVEY\SURVEY\SURVEY\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A15EE23-E9C8-402F-8BFB-5DBCB6B165C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93D295A-EA71-4C45-8E57-7D9F9C8A9B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Kết quả khảo sát đánh giá 360 / 360度評価調査結果</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>Nhận xét chung / 総合コメント</t>
+  </si>
+  <si>
+    <t>Điểm / 長所</t>
+  </si>
+  <si>
+    <t>Điểm tiêu chuẩn</t>
   </si>
 </sst>
 </file>
@@ -155,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -169,6 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -287,11 +294,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>評価シート!$N$1</c:f>
+              <c:f>評価シート!$L$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Điểm tốt / 長所</c:v>
+                  <c:v>Điểm / 長所</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -299,7 +306,7 @@
           <c:spPr>
             <a:ln w="15875" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:srgbClr val="FF0000"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -316,7 +323,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>評価シート!$M$2:$M$6</c:f>
+              <c:f>評価シート!$K$2:$K$6</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -339,7 +346,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>評価シート!$N$2:$N$6</c:f>
+              <c:f>評価シート!$L$2:$L$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -372,11 +379,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>評価シート!$O$1</c:f>
+              <c:f>評価シート!$M$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Điểm cần cải thiện / 短所</c:v>
+                  <c:v>Điểm tiêu chuẩn</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -384,7 +391,7 @@
           <c:spPr>
             <a:ln w="15875" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent2"/>
+                <a:srgbClr val="00B050"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -401,7 +408,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>評価シート!$M$2:$M$6</c:f>
+              <c:f>評価シート!$K$2:$K$6</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -424,24 +431,24 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>評価シート!$O$2:$O$6</c:f>
+              <c:f>評価シート!$M$2:$M$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -967,119 +974,109 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" style="5" customWidth="1"/>
     <col min="2" max="2" width="47.5703125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="35.42578125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="38.5703125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="51.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="15" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.42578125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="34.140625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="38.5703125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="51.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="13" max="13" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="K1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" t="s">
+        <v>17</v>
+      </c>
       <c r="M1" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="M2" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="K2" t="s">
         <v>3</v>
       </c>
-      <c r="N2">
-        <f>$C7</f>
+      <c r="L2">
+        <f>$H7</f>
         <v>0</v>
       </c>
-      <c r="O2">
-        <f>$G7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="M3" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="N3" s="7">
-        <f t="shared" ref="N3:N6" si="0">$C8</f>
+      <c r="L3" s="8">
+        <f t="shared" ref="L3:L6" si="0">$H8</f>
         <v>0</v>
       </c>
-      <c r="O3" s="7">
-        <f t="shared" ref="O3:O6" si="1">$G8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M3" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="M4" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="K4" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="7">
+      <c r="L4" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O4" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M5" t="s">
+      <c r="M4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="7">
+      <c r="L5" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O5" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M5" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -1087,39 +1084,35 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="7">
+      <c r="L6" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O6" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M6" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1130,9 +1123,8 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1143,9 +1135,8 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-    </row>
-    <row r="9" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -1156,9 +1147,8 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-    </row>
-    <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -1169,9 +1159,8 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-    </row>
-    <row r="11" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
@@ -1182,62 +1171,53 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-    </row>
-    <row r="13" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+    </row>
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="9"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A14:I16"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="A14:G16"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
sửa giao diện màn hình ghi đánh giá
</commit_message>
<xml_diff>
--- a/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
+++ b/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\khanhmf\SURVEY\SURVEY\SURVEY\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93D295A-EA71-4C45-8E57-7D9F9C8A9B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8125EE51-B57A-4F73-9E86-7C4D59EED94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
     <t>Điểm / 長所</t>
   </si>
   <si>
-    <t>Điểm tiêu chuẩn</t>
+    <t>Điểm tiêu chuẩn/ベンチマークスコア</t>
   </si>
 </sst>
 </file>
@@ -383,7 +383,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Điểm tiêu chuẩn</c:v>
+                  <c:v>Điểm tiêu chuẩn/ベンチマークスコア</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -987,7 +987,7 @@
     <col min="8" max="8" width="15.85546875" customWidth="1"/>
     <col min="11" max="11" width="51.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19" customWidth="1"/>
-    <col min="13" max="13" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
thêm điều kiện check
</commit_message>
<xml_diff>
--- a/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
+++ b/SURVEY/wwwroot/template/Formatted_Employee_Evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\khanhmf\SURVEY\SURVEY\SURVEY\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8125EE51-B57A-4F73-9E86-7C4D59EED94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{513559EC-5E89-4F17-AC39-D31D049AA284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="評価シート" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,6 @@
     <t>Kết quả khảo sát đánh giá 360 / 360度評価調査結果</t>
   </si>
   <si>
-    <t>Category</t>
-  </si>
-  <si>
     <t>Tên nhân viên / 氏名</t>
   </si>
   <si>
@@ -62,34 +59,37 @@
     <t>4. Trách nhiệm &amp; tự chủ / 責任感・主体性</t>
   </si>
   <si>
-    <t>Nhóm / 評価項目</t>
-  </si>
-  <si>
-    <t>Điểm tốt / 長所</t>
-  </si>
-  <si>
-    <t>Điểm / 評価</t>
-  </si>
-  <si>
     <t>Tình huống / 事例</t>
   </si>
   <si>
     <t>Cải tiến / 改善案</t>
   </si>
   <si>
-    <t>Điểm cần cải thiện / 短所</t>
-  </si>
-  <si>
     <t>5. Kỷ luật &amp; tuân thủ thời gian / 規律・時間遵守</t>
   </si>
   <si>
     <t>Nhận xét chung / 総合コメント</t>
   </si>
   <si>
-    <t>Điểm / 長所</t>
-  </si>
-  <si>
-    <t>Điểm tiêu chuẩn/ベンチマークスコア</t>
+    <t>Điểm tốt / 良点</t>
+  </si>
+  <si>
+    <t>Điểm cần cải thiện / 改善点</t>
+  </si>
+  <si>
+    <t>Hạng mục đánh giá / 評価項目</t>
+  </si>
+  <si>
+    <t>Hạng mục đánh giá/評価項目</t>
+  </si>
+  <si>
+    <t>Điểm tiêu chuẩn/標準スコア</t>
+  </si>
+  <si>
+    <t>Điểm được đánh giá / スコア</t>
+  </si>
+  <si>
+    <t>Điểm được đánh giá / 	スコア</t>
   </si>
 </sst>
 </file>
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -183,7 +183,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -298,7 +301,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Điểm / 長所</c:v>
+                  <c:v>Điểm được đánh giá / スコア</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -383,7 +386,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Điểm tiêu chuẩn/ベンチマークスコア</c:v>
+                  <c:v>Điểm tiêu chuẩn/標準スコア</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -984,9 +987,9 @@
     <col min="5" max="5" width="29.5703125" style="5" customWidth="1"/>
     <col min="6" max="6" width="34.140625" style="5" customWidth="1"/>
     <col min="7" max="7" width="38.5703125" style="5" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" customWidth="1"/>
     <col min="11" max="11" width="51.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="12" max="12" width="34.7109375" customWidth="1"/>
     <col min="13" max="13" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -994,31 +997,31 @@
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
       <c r="K1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="L1" t="s">
         <v>17</v>
       </c>
       <c r="M1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="K2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <f>$H7</f>
@@ -1030,13 +1033,13 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="K3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L3" s="8">
         <f t="shared" ref="L3:L6" si="0">$H8</f>
@@ -1048,13 +1051,13 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="K4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L4" s="8">
         <f t="shared" si="0"/>
@@ -1066,7 +1069,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L5" s="8">
         <f t="shared" si="0"/>
@@ -1078,31 +1081,31 @@
     </row>
     <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="L6" s="8">
         <f t="shared" si="0"/>
@@ -1114,7 +1117,7 @@
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1126,7 +1129,7 @@
     </row>
     <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1138,7 +1141,7 @@
     </row>
     <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1150,7 +1153,7 @@
     </row>
     <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1162,7 +1165,7 @@
     </row>
     <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1174,7 +1177,7 @@
     </row>
     <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>

</xml_diff>